<commit_message>
Elec updates to files for 4.0.5
</commit_message>
<xml_diff>
--- a/InputData/elec/EIaE/Elec Imports and Exports.xlsx
+++ b/InputData/elec/EIaE/Elec Imports and Exports.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\NEXT Group\90. 개인 폴더\이지우\단기대응\202501 EPS 수요전망\V3\EIaE\old\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\elec\EIaE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B55CE2-770F-447A-B869-A6B4FB0B829D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418A509C-E300-41BF-83F0-8452706F8C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2616" yWindow="2616" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="EIaE-BIE" sheetId="3" r:id="rId2"/>
     <sheet name="EIaE-BEE" sheetId="5" r:id="rId3"/>
     <sheet name="EIaE-IEP" sheetId="9" r:id="rId4"/>
-    <sheet name="EIaE-BEEP" sheetId="10" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="lignite_multiplier">'[1]Hard Coal and Lig Multipliers'!$N$16</definedName>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>EIaE BAU Imported Electricity</t>
   </si>
@@ -115,9 +114,6 @@
     <t>Unit: 2012 USD/MWh</t>
   </si>
   <si>
-    <t>Exported Electricity Price</t>
-  </si>
-  <si>
     <t>EIaE Imported Electricity Price</t>
   </si>
   <si>
@@ -160,13 +156,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -174,7 +170,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -207,13 +203,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -221,7 +217,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -299,7 +295,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyBorder="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment wrapText="1"/>
@@ -317,7 +313,7 @@
       <alignment wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -331,7 +327,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -339,20 +334,20 @@
   <cellStyles count="16">
     <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Body: normal cell 2" xfId="14" xr:uid="{51B22B8D-CF9D-46AD-BF65-4C4D416ECE20}"/>
+    <cellStyle name="Comma" xfId="9" builtinId="3"/>
     <cellStyle name="Font: Calibri, 9pt regular" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Font: Calibri, 9pt regular 2" xfId="10" xr:uid="{382B750F-5A54-4636-ADA6-0DA00478492B}"/>
     <cellStyle name="Footnotes: top row" xfId="6" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Footnotes: top row 2" xfId="15" xr:uid="{D86F4493-36AD-40FB-B8F1-3749D0EDAFD8}"/>
     <cellStyle name="Header: bottom row" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Header: bottom row 2" xfId="11" xr:uid="{D124DBBE-817F-4F9A-B086-7B91EE80FB92}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="Normal 2 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Parent row" xfId="4" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="Parent row 2" xfId="13" xr:uid="{004140A3-0A0D-4133-A16E-5D203A439566}"/>
     <cellStyle name="Table title" xfId="3" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
     <cellStyle name="Table title 2" xfId="12" xr:uid="{D271D59B-77D2-4405-AFE3-35DCF4B982EE}"/>
-    <cellStyle name="쉼표" xfId="9" builtinId="3"/>
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -368,8 +363,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="About"/>
       <sheetName val="AEO Table 2"/>
@@ -448,9 +446,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -488,9 +486,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -523,26 +521,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -575,26 +556,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -768,224 +732,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B55"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="70.19921875" customWidth="1"/>
+    <col min="2" max="2" width="70.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="7"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B7" s="7"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B9" s="7"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B10" s="7"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B11" s="7"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B12" s="7"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B13" s="7"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B14" s="7"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B15" s="7"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B16" s="7"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B17" s="7"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B18" s="7"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B19" s="7"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B20" s="7"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A42" s="7"/>
-      <c r="B42" s="7"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A48" s="7"/>
-      <c r="B48" s="7"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A49" s="7"/>
-      <c r="B49" s="7"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A50" s="7"/>
-      <c r="B50" s="7"/>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A51" s="7"/>
-      <c r="B51" s="7"/>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A52" s="7"/>
-      <c r="B52" s="7"/>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A53" s="7"/>
-      <c r="B53" s="7"/>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A55" s="7"/>
-      <c r="B55" s="7"/>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -1000,13 +784,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF25"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="26.19921875" style="2" customWidth="1"/>
-    <col min="2" max="32" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.1796875" style="2" customWidth="1"/>
+    <col min="2" max="32" width="11.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:32" ht="29">
       <c r="A1" s="4" t="s">
         <v>20</v>
       </c>
@@ -1104,7 +888,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:32">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1202,203 +986,203 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:32">
       <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
+        <v>0</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3">
+        <v>0</v>
+      </c>
+      <c r="N3" s="3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="3">
+        <v>0</v>
+      </c>
+      <c r="P3" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>0</v>
+      </c>
+      <c r="R3" s="3">
+        <v>0</v>
+      </c>
+      <c r="S3" s="3">
+        <v>0</v>
+      </c>
+      <c r="T3" s="3">
+        <v>0</v>
+      </c>
+      <c r="U3" s="3">
+        <v>0</v>
+      </c>
+      <c r="V3" s="3">
+        <v>0</v>
+      </c>
+      <c r="W3" s="3">
+        <v>0</v>
+      </c>
+      <c r="X3" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32">
+      <c r="A4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="3">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0</v>
-      </c>
-      <c r="G3" s="3">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0</v>
-      </c>
-      <c r="K3" s="3">
-        <v>0</v>
-      </c>
-      <c r="L3" s="3">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3">
-        <v>0</v>
-      </c>
-      <c r="N3" s="3">
-        <v>0</v>
-      </c>
-      <c r="O3" s="3">
-        <v>0</v>
-      </c>
-      <c r="P3" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="3">
-        <v>0</v>
-      </c>
-      <c r="R3" s="3">
-        <v>0</v>
-      </c>
-      <c r="S3" s="3">
-        <v>0</v>
-      </c>
-      <c r="T3" s="3">
-        <v>0</v>
-      </c>
-      <c r="U3" s="3">
-        <v>0</v>
-      </c>
-      <c r="V3" s="3">
-        <v>0</v>
-      </c>
-      <c r="W3" s="3">
-        <v>0</v>
-      </c>
-      <c r="X3" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="3">
+      <c r="B4" s="3">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0</v>
+      </c>
+      <c r="M4" s="3">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3">
+        <v>0</v>
+      </c>
+      <c r="P4" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>0</v>
+      </c>
+      <c r="R4" s="3">
+        <v>0</v>
+      </c>
+      <c r="S4" s="3">
+        <v>0</v>
+      </c>
+      <c r="T4" s="3">
+        <v>0</v>
+      </c>
+      <c r="U4" s="3">
+        <v>0</v>
+      </c>
+      <c r="V4" s="3">
+        <v>0</v>
+      </c>
+      <c r="W4" s="3">
+        <v>0</v>
+      </c>
+      <c r="X4" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B4" s="3">
-        <v>0</v>
-      </c>
-      <c r="C4" s="3">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>0</v>
-      </c>
-      <c r="F4" s="3">
-        <v>0</v>
-      </c>
-      <c r="G4" s="3">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3">
-        <v>0</v>
-      </c>
-      <c r="J4" s="3">
-        <v>0</v>
-      </c>
-      <c r="K4" s="3">
-        <v>0</v>
-      </c>
-      <c r="L4" s="3">
-        <v>0</v>
-      </c>
-      <c r="M4" s="3">
-        <v>0</v>
-      </c>
-      <c r="N4" s="3">
-        <v>0</v>
-      </c>
-      <c r="O4" s="3">
-        <v>0</v>
-      </c>
-      <c r="P4" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="3">
-        <v>0</v>
-      </c>
-      <c r="R4" s="3">
-        <v>0</v>
-      </c>
-      <c r="S4" s="3">
-        <v>0</v>
-      </c>
-      <c r="T4" s="3">
-        <v>0</v>
-      </c>
-      <c r="U4" s="3">
-        <v>0</v>
-      </c>
-      <c r="V4" s="3">
-        <v>0</v>
-      </c>
-      <c r="W4" s="3">
-        <v>0</v>
-      </c>
-      <c r="X4" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:32">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1496,7 +1280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:32">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -1594,7 +1378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:32">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1692,7 +1476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:32">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -1790,7 +1574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:32">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -1888,7 +1672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:32">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -1986,7 +1770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:32">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
@@ -2084,7 +1868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:32">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2182,7 +1966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:32">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -2280,7 +2064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:32">
       <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
@@ -2378,7 +2162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:32">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -2476,7 +2260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:32">
       <c r="A16" s="2" t="s">
         <v>17</v>
       </c>
@@ -2574,7 +2358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:32">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -2672,7 +2456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:32">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -2770,597 +2554,597 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:32">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="3">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3">
+        <v>0</v>
+      </c>
+      <c r="I19" s="3">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3">
+        <v>0</v>
+      </c>
+      <c r="K19" s="3">
+        <v>0</v>
+      </c>
+      <c r="L19" s="3">
+        <v>0</v>
+      </c>
+      <c r="M19" s="3">
+        <v>0</v>
+      </c>
+      <c r="N19" s="3">
+        <v>0</v>
+      </c>
+      <c r="O19" s="3">
+        <v>0</v>
+      </c>
+      <c r="P19" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>0</v>
+      </c>
+      <c r="R19" s="3">
+        <v>0</v>
+      </c>
+      <c r="S19" s="3">
+        <v>0</v>
+      </c>
+      <c r="T19" s="3">
+        <v>0</v>
+      </c>
+      <c r="U19" s="3">
+        <v>0</v>
+      </c>
+      <c r="V19" s="3">
+        <v>0</v>
+      </c>
+      <c r="W19" s="3">
+        <v>0</v>
+      </c>
+      <c r="X19" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32">
+      <c r="A20" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="3">
-        <v>0</v>
-      </c>
-      <c r="C19" s="3">
-        <v>0</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3">
-        <v>0</v>
-      </c>
-      <c r="F19" s="3">
-        <v>0</v>
-      </c>
-      <c r="G19" s="3">
-        <v>0</v>
-      </c>
-      <c r="H19" s="3">
-        <v>0</v>
-      </c>
-      <c r="I19" s="3">
-        <v>0</v>
-      </c>
-      <c r="J19" s="3">
-        <v>0</v>
-      </c>
-      <c r="K19" s="3">
-        <v>0</v>
-      </c>
-      <c r="L19" s="3">
-        <v>0</v>
-      </c>
-      <c r="M19" s="3">
-        <v>0</v>
-      </c>
-      <c r="N19" s="3">
-        <v>0</v>
-      </c>
-      <c r="O19" s="3">
-        <v>0</v>
-      </c>
-      <c r="P19" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="3">
-        <v>0</v>
-      </c>
-      <c r="R19" s="3">
-        <v>0</v>
-      </c>
-      <c r="S19" s="3">
-        <v>0</v>
-      </c>
-      <c r="T19" s="3">
-        <v>0</v>
-      </c>
-      <c r="U19" s="3">
-        <v>0</v>
-      </c>
-      <c r="V19" s="3">
-        <v>0</v>
-      </c>
-      <c r="W19" s="3">
-        <v>0</v>
-      </c>
-      <c r="X19" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE19" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF19" s="3">
+      <c r="B20" s="3">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0</v>
+      </c>
+      <c r="I20" s="3">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3">
+        <v>0</v>
+      </c>
+      <c r="L20" s="3">
+        <v>0</v>
+      </c>
+      <c r="M20" s="3">
+        <v>0</v>
+      </c>
+      <c r="N20" s="3">
+        <v>0</v>
+      </c>
+      <c r="O20" s="3">
+        <v>0</v>
+      </c>
+      <c r="P20" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>0</v>
+      </c>
+      <c r="R20" s="3">
+        <v>0</v>
+      </c>
+      <c r="S20" s="3">
+        <v>0</v>
+      </c>
+      <c r="T20" s="3">
+        <v>0</v>
+      </c>
+      <c r="U20" s="3">
+        <v>0</v>
+      </c>
+      <c r="V20" s="3">
+        <v>0</v>
+      </c>
+      <c r="W20" s="3">
+        <v>0</v>
+      </c>
+      <c r="X20" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A20" s="7" t="s">
+    <row r="21" spans="1:32">
+      <c r="A21" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="3">
-        <v>0</v>
-      </c>
-      <c r="C20" s="3">
-        <v>0</v>
-      </c>
-      <c r="D20" s="3">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3">
-        <v>0</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0</v>
-      </c>
-      <c r="G20" s="3">
-        <v>0</v>
-      </c>
-      <c r="H20" s="3">
-        <v>0</v>
-      </c>
-      <c r="I20" s="3">
-        <v>0</v>
-      </c>
-      <c r="J20" s="3">
-        <v>0</v>
-      </c>
-      <c r="K20" s="3">
-        <v>0</v>
-      </c>
-      <c r="L20" s="3">
-        <v>0</v>
-      </c>
-      <c r="M20" s="3">
-        <v>0</v>
-      </c>
-      <c r="N20" s="3">
-        <v>0</v>
-      </c>
-      <c r="O20" s="3">
-        <v>0</v>
-      </c>
-      <c r="P20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="3">
-        <v>0</v>
-      </c>
-      <c r="R20" s="3">
-        <v>0</v>
-      </c>
-      <c r="S20" s="3">
-        <v>0</v>
-      </c>
-      <c r="T20" s="3">
-        <v>0</v>
-      </c>
-      <c r="U20" s="3">
-        <v>0</v>
-      </c>
-      <c r="V20" s="3">
-        <v>0</v>
-      </c>
-      <c r="W20" s="3">
-        <v>0</v>
-      </c>
-      <c r="X20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE20" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF20" s="3">
+      <c r="B21" s="3">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3">
+        <v>0</v>
+      </c>
+      <c r="I21" s="3">
+        <v>0</v>
+      </c>
+      <c r="J21" s="3">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3">
+        <v>0</v>
+      </c>
+      <c r="L21" s="3">
+        <v>0</v>
+      </c>
+      <c r="M21" s="3">
+        <v>0</v>
+      </c>
+      <c r="N21" s="3">
+        <v>0</v>
+      </c>
+      <c r="O21" s="3">
+        <v>0</v>
+      </c>
+      <c r="P21" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>0</v>
+      </c>
+      <c r="R21" s="3">
+        <v>0</v>
+      </c>
+      <c r="S21" s="3">
+        <v>0</v>
+      </c>
+      <c r="T21" s="3">
+        <v>0</v>
+      </c>
+      <c r="U21" s="3">
+        <v>0</v>
+      </c>
+      <c r="V21" s="3">
+        <v>0</v>
+      </c>
+      <c r="W21" s="3">
+        <v>0</v>
+      </c>
+      <c r="X21" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A21" s="7" t="s">
+    <row r="22" spans="1:32">
+      <c r="A22" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="3">
-        <v>0</v>
-      </c>
-      <c r="C21" s="3">
-        <v>0</v>
-      </c>
-      <c r="D21" s="3">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3">
-        <v>0</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3">
-        <v>0</v>
-      </c>
-      <c r="I21" s="3">
-        <v>0</v>
-      </c>
-      <c r="J21" s="3">
-        <v>0</v>
-      </c>
-      <c r="K21" s="3">
-        <v>0</v>
-      </c>
-      <c r="L21" s="3">
-        <v>0</v>
-      </c>
-      <c r="M21" s="3">
-        <v>0</v>
-      </c>
-      <c r="N21" s="3">
-        <v>0</v>
-      </c>
-      <c r="O21" s="3">
-        <v>0</v>
-      </c>
-      <c r="P21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="3">
-        <v>0</v>
-      </c>
-      <c r="R21" s="3">
-        <v>0</v>
-      </c>
-      <c r="S21" s="3">
-        <v>0</v>
-      </c>
-      <c r="T21" s="3">
-        <v>0</v>
-      </c>
-      <c r="U21" s="3">
-        <v>0</v>
-      </c>
-      <c r="V21" s="3">
-        <v>0</v>
-      </c>
-      <c r="W21" s="3">
-        <v>0</v>
-      </c>
-      <c r="X21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y21" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE21" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF21" s="3">
+      <c r="B22" s="3">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3">
+        <v>0</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3">
+        <v>0</v>
+      </c>
+      <c r="L22" s="3">
+        <v>0</v>
+      </c>
+      <c r="M22" s="3">
+        <v>0</v>
+      </c>
+      <c r="N22" s="3">
+        <v>0</v>
+      </c>
+      <c r="O22" s="3">
+        <v>0</v>
+      </c>
+      <c r="P22" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="3">
+        <v>0</v>
+      </c>
+      <c r="R22" s="3">
+        <v>0</v>
+      </c>
+      <c r="S22" s="3">
+        <v>0</v>
+      </c>
+      <c r="T22" s="3">
+        <v>0</v>
+      </c>
+      <c r="U22" s="3">
+        <v>0</v>
+      </c>
+      <c r="V22" s="3">
+        <v>0</v>
+      </c>
+      <c r="W22" s="3">
+        <v>0</v>
+      </c>
+      <c r="X22" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A22" s="7" t="s">
+    <row r="23" spans="1:32">
+      <c r="A23" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="3">
-        <v>0</v>
-      </c>
-      <c r="C22" s="3">
-        <v>0</v>
-      </c>
-      <c r="D22" s="3">
-        <v>0</v>
-      </c>
-      <c r="E22" s="3">
-        <v>0</v>
-      </c>
-      <c r="F22" s="3">
-        <v>0</v>
-      </c>
-      <c r="G22" s="3">
-        <v>0</v>
-      </c>
-      <c r="H22" s="3">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3">
-        <v>0</v>
-      </c>
-      <c r="J22" s="3">
-        <v>0</v>
-      </c>
-      <c r="K22" s="3">
-        <v>0</v>
-      </c>
-      <c r="L22" s="3">
-        <v>0</v>
-      </c>
-      <c r="M22" s="3">
-        <v>0</v>
-      </c>
-      <c r="N22" s="3">
-        <v>0</v>
-      </c>
-      <c r="O22" s="3">
-        <v>0</v>
-      </c>
-      <c r="P22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="3">
-        <v>0</v>
-      </c>
-      <c r="R22" s="3">
-        <v>0</v>
-      </c>
-      <c r="S22" s="3">
-        <v>0</v>
-      </c>
-      <c r="T22" s="3">
-        <v>0</v>
-      </c>
-      <c r="U22" s="3">
-        <v>0</v>
-      </c>
-      <c r="V22" s="3">
-        <v>0</v>
-      </c>
-      <c r="W22" s="3">
-        <v>0</v>
-      </c>
-      <c r="X22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE22" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF22" s="3">
+      <c r="B23" s="3">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3">
+        <v>0</v>
+      </c>
+      <c r="L23" s="3">
+        <v>0</v>
+      </c>
+      <c r="M23" s="3">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3">
+        <v>0</v>
+      </c>
+      <c r="O23" s="3">
+        <v>0</v>
+      </c>
+      <c r="P23" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="3">
+        <v>0</v>
+      </c>
+      <c r="R23" s="3">
+        <v>0</v>
+      </c>
+      <c r="S23" s="3">
+        <v>0</v>
+      </c>
+      <c r="T23" s="3">
+        <v>0</v>
+      </c>
+      <c r="U23" s="3">
+        <v>0</v>
+      </c>
+      <c r="V23" s="3">
+        <v>0</v>
+      </c>
+      <c r="W23" s="3">
+        <v>0</v>
+      </c>
+      <c r="X23" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A23" s="7" t="s">
+    <row r="24" spans="1:32">
+      <c r="A24" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="3">
-        <v>0</v>
-      </c>
-      <c r="C23" s="3">
-        <v>0</v>
-      </c>
-      <c r="D23" s="3">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3">
-        <v>0</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="3">
-        <v>0</v>
-      </c>
-      <c r="H23" s="3">
-        <v>0</v>
-      </c>
-      <c r="I23" s="3">
-        <v>0</v>
-      </c>
-      <c r="J23" s="3">
-        <v>0</v>
-      </c>
-      <c r="K23" s="3">
-        <v>0</v>
-      </c>
-      <c r="L23" s="3">
-        <v>0</v>
-      </c>
-      <c r="M23" s="3">
-        <v>0</v>
-      </c>
-      <c r="N23" s="3">
-        <v>0</v>
-      </c>
-      <c r="O23" s="3">
-        <v>0</v>
-      </c>
-      <c r="P23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="3">
-        <v>0</v>
-      </c>
-      <c r="R23" s="3">
-        <v>0</v>
-      </c>
-      <c r="S23" s="3">
-        <v>0</v>
-      </c>
-      <c r="T23" s="3">
-        <v>0</v>
-      </c>
-      <c r="U23" s="3">
-        <v>0</v>
-      </c>
-      <c r="V23" s="3">
-        <v>0</v>
-      </c>
-      <c r="W23" s="3">
-        <v>0</v>
-      </c>
-      <c r="X23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE23" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF23" s="3">
+      <c r="B24" s="3">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0</v>
+      </c>
+      <c r="H24" s="3">
+        <v>0</v>
+      </c>
+      <c r="I24" s="3">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3">
+        <v>0</v>
+      </c>
+      <c r="L24" s="3">
+        <v>0</v>
+      </c>
+      <c r="M24" s="3">
+        <v>0</v>
+      </c>
+      <c r="N24" s="3">
+        <v>0</v>
+      </c>
+      <c r="O24" s="3">
+        <v>0</v>
+      </c>
+      <c r="P24" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="3">
+        <v>0</v>
+      </c>
+      <c r="R24" s="3">
+        <v>0</v>
+      </c>
+      <c r="S24" s="3">
+        <v>0</v>
+      </c>
+      <c r="T24" s="3">
+        <v>0</v>
+      </c>
+      <c r="U24" s="3">
+        <v>0</v>
+      </c>
+      <c r="V24" s="3">
+        <v>0</v>
+      </c>
+      <c r="W24" s="3">
+        <v>0</v>
+      </c>
+      <c r="X24" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF24" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A24" s="8" t="s">
+    <row r="25" spans="1:32">
+      <c r="A25" s="7" t="s">
         <v>35</v>
-      </c>
-      <c r="B24" s="3">
-        <v>0</v>
-      </c>
-      <c r="C24" s="3">
-        <v>0</v>
-      </c>
-      <c r="D24" s="3">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3">
-        <v>0</v>
-      </c>
-      <c r="F24" s="3">
-        <v>0</v>
-      </c>
-      <c r="G24" s="3">
-        <v>0</v>
-      </c>
-      <c r="H24" s="3">
-        <v>0</v>
-      </c>
-      <c r="I24" s="3">
-        <v>0</v>
-      </c>
-      <c r="J24" s="3">
-        <v>0</v>
-      </c>
-      <c r="K24" s="3">
-        <v>0</v>
-      </c>
-      <c r="L24" s="3">
-        <v>0</v>
-      </c>
-      <c r="M24" s="3">
-        <v>0</v>
-      </c>
-      <c r="N24" s="3">
-        <v>0</v>
-      </c>
-      <c r="O24" s="3">
-        <v>0</v>
-      </c>
-      <c r="P24" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="3">
-        <v>0</v>
-      </c>
-      <c r="R24" s="3">
-        <v>0</v>
-      </c>
-      <c r="S24" s="3">
-        <v>0</v>
-      </c>
-      <c r="T24" s="3">
-        <v>0</v>
-      </c>
-      <c r="U24" s="3">
-        <v>0</v>
-      </c>
-      <c r="V24" s="3">
-        <v>0</v>
-      </c>
-      <c r="W24" s="3">
-        <v>0</v>
-      </c>
-      <c r="X24" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE24" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF24" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.4">
-      <c r="A25" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="B25" s="3">
         <v>0</v>
@@ -3468,12 +3252,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="26.19921875" customWidth="1"/>
+    <col min="1" max="1" width="26.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:32" ht="29">
       <c r="A1" s="5" t="s">
         <v>21</v>
       </c>
@@ -3571,101 +3355,101 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:32">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" s="7">
-        <v>0</v>
-      </c>
-      <c r="D2" s="7">
-        <v>0</v>
-      </c>
-      <c r="E2" s="7">
-        <v>0</v>
-      </c>
-      <c r="F2" s="7">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7">
-        <v>0</v>
-      </c>
-      <c r="J2" s="7">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7">
-        <v>0</v>
-      </c>
-      <c r="N2" s="7">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7">
-        <v>0</v>
-      </c>
-      <c r="P2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="7">
-        <v>0</v>
-      </c>
-      <c r="R2" s="7">
-        <v>0</v>
-      </c>
-      <c r="S2" s="7">
-        <v>0</v>
-      </c>
-      <c r="T2" s="7">
-        <v>0</v>
-      </c>
-      <c r="U2" s="7">
-        <v>0</v>
-      </c>
-      <c r="V2" s="7">
-        <v>0</v>
-      </c>
-      <c r="W2" s="7">
-        <v>0</v>
-      </c>
-      <c r="X2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="7">
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
         <v>0</v>
       </c>
     </row>
@@ -3681,12 +3465,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="26.19921875" customWidth="1"/>
+    <col min="1" max="1" width="26.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:34">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
@@ -3784,225 +3568,9 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:34">
       <c r="A2" t="s">
         <v>22</v>
-      </c>
-      <c r="B2" s="6">
-        <v>0</v>
-      </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6">
-        <v>0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6">
-        <v>0</v>
-      </c>
-      <c r="G2" s="6">
-        <v>0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0</v>
-      </c>
-      <c r="J2" s="6">
-        <v>0</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
-        <v>0</v>
-      </c>
-      <c r="U2" s="6">
-        <v>0</v>
-      </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="6"/>
-      <c r="AH2" s="6"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{364777A9-21C3-491A-80BE-AFAA838DFA2A}">
-  <sheetPr>
-    <tabColor theme="3"/>
-  </sheetPr>
-  <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="26.19921875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="A1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1">
-        <v>2020</v>
-      </c>
-      <c r="C1">
-        <v>2021</v>
-      </c>
-      <c r="D1">
-        <v>2022</v>
-      </c>
-      <c r="E1">
-        <v>2023</v>
-      </c>
-      <c r="F1">
-        <v>2024</v>
-      </c>
-      <c r="G1">
-        <v>2025</v>
-      </c>
-      <c r="H1">
-        <v>2026</v>
-      </c>
-      <c r="I1">
-        <v>2027</v>
-      </c>
-      <c r="J1">
-        <v>2028</v>
-      </c>
-      <c r="K1">
-        <v>2029</v>
-      </c>
-      <c r="L1">
-        <v>2030</v>
-      </c>
-      <c r="M1">
-        <v>2031</v>
-      </c>
-      <c r="N1">
-        <v>2032</v>
-      </c>
-      <c r="O1">
-        <v>2033</v>
-      </c>
-      <c r="P1">
-        <v>2034</v>
-      </c>
-      <c r="Q1">
-        <v>2035</v>
-      </c>
-      <c r="R1">
-        <v>2036</v>
-      </c>
-      <c r="S1">
-        <v>2037</v>
-      </c>
-      <c r="T1">
-        <v>2038</v>
-      </c>
-      <c r="U1">
-        <v>2039</v>
-      </c>
-      <c r="V1">
-        <v>2040</v>
-      </c>
-      <c r="W1">
-        <v>2041</v>
-      </c>
-      <c r="X1">
-        <v>2042</v>
-      </c>
-      <c r="Y1">
-        <v>2043</v>
-      </c>
-      <c r="Z1">
-        <v>2044</v>
-      </c>
-      <c r="AA1">
-        <v>2045</v>
-      </c>
-      <c r="AB1">
-        <v>2046</v>
-      </c>
-      <c r="AC1">
-        <v>2047</v>
-      </c>
-      <c r="AD1">
-        <v>2048</v>
-      </c>
-      <c r="AE1">
-        <v>2049</v>
-      </c>
-      <c r="AF1">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>24</v>
       </c>
       <c r="B2" s="6">
         <v>0</v>
@@ -4108,6 +3676,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -4251,15 +3828,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -4267,13 +3835,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65E49E72-0524-4344-A2FC-5EE44029CC1F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6A66BB2-46C1-4E6C-AAD2-49F519ECFAF5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6A66BB2-46C1-4E6C-AAD2-49F519ECFAF5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65E49E72-0524-4344-A2FC-5EE44029CC1F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54617A8D-0AFE-4BAE-A70E-BCCC84E48339}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54617A8D-0AFE-4BAE-A70E-BCCC84E48339}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>